<commit_message>
Initial commit - OrthoLegal Test Automation PY
</commit_message>
<xml_diff>
--- a/test_data/PQME_Encounter_Test_Data.xlsx
+++ b/test_data/PQME_Encounter_Test_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rishi Files\OrthoLegal_Automation\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B521AA1F-2FC3-4214-9365-E7382A67FD5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76E84B68-21C1-4209-BEB6-E378DB1A9EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="1092" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Encounter_Test_Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="117">
   <si>
     <t>Applicant Details</t>
   </si>
@@ -196,15 +196,6 @@
     <t>Adjuster Assistant Email</t>
   </si>
   <si>
-    <t>ANeoers</t>
-  </si>
-  <si>
-    <t>Devtest</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
     <t>Male</t>
   </si>
   <si>
@@ -374,6 +365,12 @@
   </si>
   <si>
     <t>(714) 555-2389</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Kumar</t>
   </si>
 </sst>
 </file>
@@ -1256,73 +1253,73 @@
     </row>
     <row r="3" spans="1:87" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="3">
+        <v>36608</v>
+      </c>
+      <c r="E3" t="s">
         <v>58</v>
       </c>
-      <c r="B3" t="s">
+      <c r="F3" t="s">
         <v>59</v>
       </c>
-      <c r="C3" t="s">
+      <c r="G3" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="3">
-        <v>31758</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="H3" t="s">
         <v>61</v>
       </c>
-      <c r="F3" t="s">
+      <c r="I3" t="s">
         <v>62</v>
       </c>
-      <c r="G3" t="s">
+      <c r="J3" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="H3" t="s">
-        <v>64</v>
-      </c>
-      <c r="I3" t="s">
-        <v>65</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="K3">
         <v>94612</v>
       </c>
       <c r="L3" t="s">
+        <v>64</v>
+      </c>
+      <c r="M3" t="s">
+        <v>65</v>
+      </c>
+      <c r="N3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O3" t="s">
         <v>67</v>
       </c>
-      <c r="M3" t="s">
+      <c r="P3" t="s">
         <v>68</v>
       </c>
-      <c r="N3" t="s">
+      <c r="Q3" t="s">
         <v>69</v>
       </c>
-      <c r="O3" t="s">
+      <c r="R3" t="s">
         <v>70</v>
       </c>
-      <c r="P3" t="s">
+      <c r="S3" t="s">
         <v>71</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="T3" t="s">
         <v>72</v>
       </c>
-      <c r="R3" t="s">
+      <c r="U3" t="s">
         <v>73</v>
       </c>
-      <c r="S3" t="s">
+      <c r="V3" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="T3" t="s">
+      <c r="W3" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="U3" t="s">
-        <v>76</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="W3" s="4" t="s">
-        <v>78</v>
       </c>
       <c r="X3" s="4">
         <v>10000000000</v>
@@ -1334,16 +1331,16 @@
         <v>46335.416666666664</v>
       </c>
       <c r="AA3" s="4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="AB3" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="AC3" s="4" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="AD3" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="AE3" s="4">
         <v>92626</v>
@@ -1352,163 +1349,163 @@
       <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
       <c r="AI3" s="8" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="AJ3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="AK3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="AL3" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>80</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AO3" t="s">
         <v>82</v>
       </c>
-      <c r="AM3" t="s">
+      <c r="AP3" t="s">
         <v>83</v>
       </c>
-      <c r="AN3" t="s">
+      <c r="AQ3" t="s">
         <v>84</v>
       </c>
-      <c r="AO3" t="s">
+      <c r="AR3" t="s">
         <v>85</v>
       </c>
-      <c r="AP3" t="s">
-        <v>86</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>87</v>
-      </c>
-      <c r="AR3" t="s">
-        <v>88</v>
-      </c>
       <c r="AS3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="AT3">
         <v>90001</v>
       </c>
       <c r="AU3" t="s">
+        <v>86</v>
+      </c>
+      <c r="AV3" t="s">
+        <v>87</v>
+      </c>
+      <c r="AW3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AX3" t="s">
         <v>89</v>
       </c>
-      <c r="AV3" t="s">
+      <c r="AY3" t="s">
         <v>90</v>
       </c>
-      <c r="AW3" t="s">
+      <c r="AZ3" t="s">
         <v>91</v>
       </c>
-      <c r="AX3" t="s">
+      <c r="BA3" t="s">
         <v>92</v>
       </c>
-      <c r="AY3" t="s">
-        <v>93</v>
-      </c>
-      <c r="AZ3" t="s">
-        <v>94</v>
-      </c>
-      <c r="BA3" t="s">
-        <v>95</v>
-      </c>
       <c r="BB3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="BC3" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="BD3">
         <v>90001</v>
       </c>
       <c r="BE3" t="s">
+        <v>93</v>
+      </c>
+      <c r="BF3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BG3" t="s">
+        <v>95</v>
+      </c>
+      <c r="BH3" t="s">
         <v>96</v>
       </c>
-      <c r="BF3" t="s">
+      <c r="BI3" t="s">
         <v>97</v>
       </c>
-      <c r="BG3" t="s">
+      <c r="BJ3" t="s">
         <v>98</v>
       </c>
-      <c r="BH3" t="s">
+      <c r="BK3" t="s">
         <v>99</v>
       </c>
-      <c r="BI3" t="s">
+      <c r="BL3" t="s">
+        <v>91</v>
+      </c>
+      <c r="BM3" t="s">
         <v>100</v>
       </c>
-      <c r="BJ3" t="s">
-        <v>101</v>
-      </c>
-      <c r="BK3" t="s">
-        <v>102</v>
-      </c>
-      <c r="BL3" t="s">
-        <v>94</v>
-      </c>
-      <c r="BM3" t="s">
-        <v>103</v>
-      </c>
       <c r="BN3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="BO3" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="BP3">
         <v>90001</v>
       </c>
       <c r="BQ3" t="s">
+        <v>101</v>
+      </c>
+      <c r="BR3" t="s">
+        <v>102</v>
+      </c>
+      <c r="BS3" t="s">
+        <v>103</v>
+      </c>
+      <c r="BT3" t="s">
         <v>104</v>
       </c>
-      <c r="BR3" t="s">
+      <c r="BU3" t="s">
         <v>105</v>
       </c>
-      <c r="BS3" t="s">
+      <c r="BV3" t="s">
         <v>106</v>
       </c>
-      <c r="BT3" t="s">
+      <c r="BW3" t="s">
         <v>107</v>
       </c>
-      <c r="BU3" t="s">
+      <c r="BX3" t="s">
+        <v>80</v>
+      </c>
+      <c r="BY3" t="s">
         <v>108</v>
       </c>
-      <c r="BV3" t="s">
+      <c r="BZ3" t="s">
         <v>109</v>
       </c>
-      <c r="BW3" t="s">
-        <v>110</v>
-      </c>
-      <c r="BX3" t="s">
-        <v>83</v>
-      </c>
-      <c r="BY3" t="s">
-        <v>111</v>
-      </c>
-      <c r="BZ3" t="s">
-        <v>112</v>
-      </c>
       <c r="CA3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="CB3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="CC3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="CD3" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="CE3">
         <v>90001</v>
       </c>
       <c r="CF3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="CG3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="CH3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="CI3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:87" x14ac:dyDescent="0.25">

</xml_diff>